<commit_message>
Scrub remaining firm lockup from Mac-openable Boca CLIENT xlsx.
Keep the xlsxwriter package (relative worksheet Targets). Owner's
representative is Landis Kauffman and Claudia Mardones by name only.
HTML and PDFs untouched.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
@@ -60,7 +60,7 @@
     <t>Owner's representative</t>
   </si>
   <si>
-    <t>Charrette MG — Landis Kauffman, Claudia Mardones</t>
+    <t>Landis Kauffman, Claudia Mardones</t>
   </si>
   <si>
     <t>Contract</t>
@@ -123,7 +123,7 @@
     <t>Open book</t>
   </si>
   <si>
-    <t>Preliminary open-book CM exhibit for Charrette review. Not a lump-sum bid and not an awarded contract price.</t>
+    <t>Preliminary open-book CM exhibit. Not a lump-sum bid and not an awarded contract price.</t>
   </si>
   <si>
     <t>Set vs open</t>

</xml_diff>

<commit_message>
Lock Boca SF at 3,800 and ship Landis CLIENT pack.
Replace the thin RATES workbook and the 3,384 mall-fee figure with the
Luke/Ricky-approved Landis workbook (COVER, LANDIS FORM, GC BID FORM,
MALL FEES, PROPOSED ROSTER) at 3,800 sf. Page meta and mall-fees copy
use total sf only. Pack zip rebuilt with cash PDF and CM redline.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
@@ -940,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E27"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -950,6 +950,7 @@
     <col width="18" customWidth="1" style="73" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="73">
       <c r="B2" s="78" t="inlineStr">
         <is>
@@ -971,6 +972,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="20" customHeight="1" s="73">
       <c r="B6" s="75" t="inlineStr">
         <is>
@@ -1014,7 +1016,7 @@
       </c>
       <c r="C9" s="70" t="inlineStr">
         <is>
-          <t>3,384 sf</t>
+          <t>3,800 sf</t>
         </is>
       </c>
       <c r="D9" s="94" t="n"/>
@@ -1160,6 +1162,7 @@
       <c r="D19" s="94" t="n"/>
       <c r="E19" s="95" t="n"/>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="76" t="inlineStr">
         <is>
@@ -1299,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:G48"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -1321,7 +1324,7 @@
     <row r="2" ht="28" customHeight="1" s="73">
       <c r="B2" s="83" t="inlineStr">
         <is>
-          <t>LUX Brand Company  |  Cost-plus CM + GC (open book, not lump sum)  |  Town Center at Boca Raton, Simon space 1062, 600 Glades Road  |  3,384 sf</t>
+          <t>LUX Brand Company  |  Cost-plus CM + GC (open book, not lump sum)  |  Town Center at Boca Raton, Simon space 1062, 600 Glades Road  |  3,800 sf</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:K79"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -1895,6 +1898,7 @@
     <col width="72" customWidth="1" style="73" min="11" max="11"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -1902,6 +1906,11 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8" ht="18" customHeight="1" s="73">
       <c r="I8" s="5" t="inlineStr">
         <is>
@@ -1916,6 +1925,9 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="15.75" customHeight="1" s="73">
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -2027,6 +2039,8 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
+    <row r="20"/>
     <row r="21" ht="27.75" customHeight="1" s="73">
       <c r="A21" s="16" t="n"/>
       <c r="B21" s="16" t="inlineStr">
@@ -2213,6 +2227,7 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="82" t="inlineStr">
         <is>
@@ -2229,6 +2244,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" s="80" t="inlineStr">
         <is>
@@ -2278,6 +2294,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="B34" s="80" t="inlineStr">
         <is>
@@ -2379,6 +2396,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="B39" s="80" t="inlineStr">
         <is>
@@ -2734,6 +2752,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="B51" s="80" t="inlineStr">
         <is>
@@ -3285,6 +3304,9 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
     <row r="79">
       <c r="D79" s="80" t="inlineStr">
         <is>
@@ -3361,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:H18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -3374,7 +3396,7 @@
     <row r="1" ht="24" customHeight="1" s="73">
       <c r="B1" s="78" t="inlineStr">
         <is>
-          <t>Mall fees — unit rates on 3,384 sf (notes, not a job grand total)</t>
+          <t>Mall fees — unit rates on 3,800 sf (notes, not a job grand total)</t>
         </is>
       </c>
     </row>
@@ -3385,6 +3407,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="39" t="inlineStr">
         <is>
@@ -3392,7 +3415,7 @@
         </is>
       </c>
       <c r="C4" s="56" t="n">
-        <v>3384</v>
+        <v>3800</v>
       </c>
       <c r="D4" s="93" t="inlineStr">
         <is>
@@ -3400,6 +3423,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="73">
       <c r="B6" s="42" t="inlineStr">
         <is>
@@ -3452,7 +3476,7 @@
         </is>
       </c>
       <c r="E7" s="58" t="n">
-        <v>3384</v>
+        <v>3800</v>
       </c>
       <c r="F7" s="96" t="n">
         <v>1455.12</v>
@@ -3464,7 +3488,7 @@
       </c>
       <c r="H7" s="60" t="inlineStr">
         <is>
-          <t>Unit rate $0.43/sf × 3,384 sf. Extension is rate × sf, not a job total.</t>
+          <t>Unit rate $0.43/sf × 3,800 sf. Extension is rate × sf, not a job total.</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3507,7 @@
         </is>
       </c>
       <c r="E8" s="58" t="n">
-        <v>3384</v>
+        <v>3800</v>
       </c>
       <c r="F8" s="96" t="n">
         <v>338.4</v>
@@ -3495,7 +3519,7 @@
       </c>
       <c r="H8" s="60" t="inlineStr">
         <is>
-          <t>Unit rate $0.10/sf × 3,384 sf. Extension is rate × sf, not a job total.</t>
+          <t>Unit rate $0.10/sf × 3,800 sf. Extension is rate × sf, not a job total.</t>
         </is>
       </c>
     </row>
@@ -3623,6 +3647,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="63" t="inlineStr">
         <is>
@@ -3657,10 +3682,11 @@
       <c r="G15" s="94" t="n"/>
       <c r="H15" s="95" t="n"/>
     </row>
+    <row r="16"/>
     <row r="17" ht="20" customHeight="1" s="73">
       <c r="B17" s="92" t="inlineStr">
         <is>
-          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,455.12 + temp water $338.40 + after hours $400 + tenant coordination $250 = $2,443.52. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,384 sf — not a bid total.</t>
+          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,455.12 + temp water $338.40 + after hours $400 + tenant coordination $250 = $2,443.52. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,800 sf — not a bid total.</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:E27"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -3719,6 +3745,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1" s="73">
       <c r="B4" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Boca mall-fee extensions to 0.43×3800 and 0.10×3800.
Area was already 3,800; cached temp-electric/water dollars still
used the old 3,384 sf. Set extensions to $1,634 and $380 and
update the MALL FEES rollup note. Pack zip rebuilt.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
@@ -3479,7 +3479,7 @@
         <v>3800</v>
       </c>
       <c r="F7" s="96" t="n">
-        <v>1455.12</v>
+        <v>1634</v>
       </c>
       <c r="G7" s="59" t="inlineStr">
         <is>
@@ -3510,7 +3510,7 @@
         <v>3800</v>
       </c>
       <c r="F8" s="96" t="n">
-        <v>338.4</v>
+        <v>380</v>
       </c>
       <c r="G8" s="59" t="inlineStr">
         <is>
@@ -3686,7 +3686,7 @@
     <row r="17" ht="20" customHeight="1" s="73">
       <c r="B17" s="92" t="inlineStr">
         <is>
-          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,455.12 + temp water $338.40 + after hours $400 + tenant coordination $250 = $2,443.52. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,800 sf — not a bid total.</t>
+          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,634.00 + temp water $380.00 + after hours $400 + tenant coordination $250 = $2,664.00. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,800 sf — not a bid total.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore Luke-approved Landis CLIENT workbook bytes.
Overwrite CLIENT xlsx with the verified Landis file
(md5 d38dff3793d82ec3b215f440834f0a46; COVER, LANDIS FORM,
GC BID FORM, MALL FEES, PROPOSED ROSTER) and rebuild the pack zip.

Co-authored-by: lucasoffice <lucasoffice@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
+++ b/ralph-lauren/boca/RL_Boca_CostPlus_CLIENT_2026-09-04.xlsx
@@ -940,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="B2:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -950,7 +950,6 @@
     <col width="18" customWidth="1" style="73" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="73">
       <c r="B2" s="78" t="inlineStr">
         <is>
@@ -972,7 +971,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="20" customHeight="1" s="73">
       <c r="B6" s="75" t="inlineStr">
         <is>
@@ -1016,7 +1014,7 @@
       </c>
       <c r="C9" s="70" t="inlineStr">
         <is>
-          <t>3,800 sf</t>
+          <t>3,384 sf</t>
         </is>
       </c>
       <c r="D9" s="94" t="n"/>
@@ -1162,7 +1160,6 @@
       <c r="D19" s="94" t="n"/>
       <c r="E19" s="95" t="n"/>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="76" t="inlineStr">
         <is>
@@ -1302,7 +1299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="B1:G48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -1324,7 +1321,7 @@
     <row r="2" ht="28" customHeight="1" s="73">
       <c r="B2" s="83" t="inlineStr">
         <is>
-          <t>LUX Brand Company  |  Cost-plus CM + GC (open book, not lump sum)  |  Town Center at Boca Raton, Simon space 1062, 600 Glades Road  |  3,800 sf</t>
+          <t>LUX Brand Company  |  Cost-plus CM + GC (open book, not lump sum)  |  Town Center at Boca Raton, Simon space 1062, 600 Glades Road  |  3,384 sf</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A2:K79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -1898,7 +1895,6 @@
     <col width="72" customWidth="1" style="73" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -1906,11 +1902,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8" ht="18" customHeight="1" s="73">
       <c r="I8" s="5" t="inlineStr">
         <is>
@@ -1925,9 +1916,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="15.75" customHeight="1" s="73">
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -2039,8 +2027,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21" ht="27.75" customHeight="1" s="73">
       <c r="A21" s="16" t="n"/>
       <c r="B21" s="16" t="inlineStr">
@@ -2227,7 +2213,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="B29" s="82" t="inlineStr">
         <is>
@@ -2244,7 +2229,6 @@
         <v/>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="B31" s="80" t="inlineStr">
         <is>
@@ -2294,7 +2278,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="B34" s="80" t="inlineStr">
         <is>
@@ -2396,7 +2379,6 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="B39" s="80" t="inlineStr">
         <is>
@@ -2752,7 +2734,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="B51" s="80" t="inlineStr">
         <is>
@@ -3300,13 +3281,10 @@
       </c>
       <c r="K75" s="72" t="inlineStr">
         <is>
-          <t>Listed mall unit rates (see MALL FEES): temp electric $1,634.00 + temp water $380.00 + after hours $400 + tenant coordination $250 = $2,664.00. This line stays $0 until entered as a bid dollar. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Mall figures are unit-rate notes, not a bid total.</t>
-        </is>
-      </c>
-    </row>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
+          <t>Listed mall unit rates (see MALL FEES): temp electric $1,455.12 + temp water $338.40 + after hours $400 + tenant coordination $250 = $2,443.52. This line stays $0 until entered as a bid dollar. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Mall figures are unit-rate notes, not a bid total.</t>
+        </is>
+      </c>
+    </row>
     <row r="79">
       <c r="D79" s="80" t="inlineStr">
         <is>
@@ -3383,7 +3361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="B1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -3396,7 +3374,7 @@
     <row r="1" ht="24" customHeight="1" s="73">
       <c r="B1" s="78" t="inlineStr">
         <is>
-          <t>Mall fees — unit rates on 3,800 sf (notes, not a job grand total)</t>
+          <t>Mall fees — unit rates on 3,384 sf (notes, not a job grand total)</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3385,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="39" t="inlineStr">
         <is>
@@ -3415,7 +3392,7 @@
         </is>
       </c>
       <c r="C4" s="56" t="n">
-        <v>3800</v>
+        <v>3384</v>
       </c>
       <c r="D4" s="93" t="inlineStr">
         <is>
@@ -3423,7 +3400,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="73">
       <c r="B6" s="42" t="inlineStr">
         <is>
@@ -3476,10 +3452,10 @@
         </is>
       </c>
       <c r="E7" s="58" t="n">
-        <v>3800</v>
+        <v>3384</v>
       </c>
       <c r="F7" s="96" t="n">
-        <v>1634</v>
+        <v>1455.12</v>
       </c>
       <c r="G7" s="59" t="inlineStr">
         <is>
@@ -3488,7 +3464,7 @@
       </c>
       <c r="H7" s="60" t="inlineStr">
         <is>
-          <t>Unit rate $0.43/sf × 3,800 sf. Extension is rate × sf, not a job total.</t>
+          <t>Unit rate $0.43/sf × 3,384 sf. Extension is rate × sf, not a job total.</t>
         </is>
       </c>
     </row>
@@ -3507,10 +3483,10 @@
         </is>
       </c>
       <c r="E8" s="58" t="n">
-        <v>3800</v>
+        <v>3384</v>
       </c>
       <c r="F8" s="96" t="n">
-        <v>380</v>
+        <v>338.4</v>
       </c>
       <c r="G8" s="59" t="inlineStr">
         <is>
@@ -3519,7 +3495,7 @@
       </c>
       <c r="H8" s="60" t="inlineStr">
         <is>
-          <t>Unit rate $0.10/sf × 3,800 sf. Extension is rate × sf, not a job total.</t>
+          <t>Unit rate $0.10/sf × 3,384 sf. Extension is rate × sf, not a job total.</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3623,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="63" t="inlineStr">
         <is>
@@ -3682,11 +3657,10 @@
       <c r="G15" s="94" t="n"/>
       <c r="H15" s="95" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="20" customHeight="1" s="73">
       <c r="B17" s="92" t="inlineStr">
         <is>
-          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,634.00 + temp water $380.00 + after hours $400 + tenant coordination $250 = $2,664.00. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,800 sf — not a bid total.</t>
+          <t>Listed mall dollars on this sheet (not a job grand total): temp electric $1,455.12 + temp water $338.40 + after hours $400 + tenant coordination $250 = $2,443.52. Parking months and sprinkler-shutdown count are OPEN — to be confirmed. Unit rates on 3,384 sf — not a bid total.</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" style="73" min="1" max="1"/>
@@ -3745,7 +3719,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16" customHeight="1" s="73">
       <c r="B4" s="42" t="inlineStr">
         <is>

</xml_diff>